<commit_message>
Pruebas 12/10/2026: accesibilidad y casos de correo
Repetidos CA-RNF06-1 y CA-RNF06-2 con letra al máximo y probado
CA-RNF06-3 (claro y oscuro). Casos de correo en la beta con
ojoalbondi.app@gmail.com: CA-RF02-5, CA-RF02-6, CA-RF05-3 y CA-RF02-3.
Los 7 pasan. Plan de pruebas actualizado y capturas en pruebas/capturas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
+++ b/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
@@ -894,7 +894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="20" min="1" max="1"/>
@@ -1478,10 +1478,24 @@
         </is>
       </c>
       <c r="J9" s="32" t="n"/>
-      <c r="K9" s="30" t="n"/>
-      <c r="L9" s="30" t="n"/>
-      <c r="M9" s="30" t="n"/>
-      <c r="N9" s="31" t="n"/>
+      <c r="K9" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L9" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 en la beta con ojoalbondi.app@gmail.com (en lugar de vecino1, para poder ver el mail). Con el correo vacío, la app mostró "Escribí tu correo arriba y tocá de nuevo “¿Olvidaste tu contraseña?”." Con el correo escrito mostró "Revisá tu correo — Te enviamos un mail a ojoalbondi.app@gmail.com para restablecer tu contraseña." y el mail llegó (confirmado por el equipo). No apareció el aviso de demasiados correos. Captura: correo vacío a la izquierda y envío a la derecha. No se abrió el enlace; probablemente redirija a localhost:3000 como el de confirmación (ver CA-RF02-6).</t>
+        </is>
+      </c>
+      <c r="M9" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N9" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="10" ht="23.85" customHeight="1" s="21">
       <c r="A10" s="28" t="n">
@@ -2260,10 +2274,24 @@
         </is>
       </c>
       <c r="J24" s="28" t="n"/>
-      <c r="K24" s="30" t="n"/>
-      <c r="L24" s="30" t="n"/>
-      <c r="M24" s="30" t="n"/>
-      <c r="N24" s="31" t="n"/>
+      <c r="K24" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L24" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 en la beta con ojoalbondi.app@gmail.com, cuenta nueva sin reclamos: Mis reportes muestra "Todavía no hiciste ningún reporte. Tocá "Reportar" abajo para crear el primero." (Reportar también muestra "Todavía no hiciste ningún reporte.").</t>
+        </is>
+      </c>
+      <c r="M24" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N24" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1" s="21">
       <c r="A25" s="32" t="n">
@@ -4108,21 +4136,21 @@
       </c>
       <c r="K56" s="30" t="inlineStr">
         <is>
-          <t>Falla</t>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L56" s="30" t="inlineStr">
         <is>
-          <t>Repetida el 11/10/2026 con letra del sistema al máximo (font_scale 2.0); recorrí Bienvenida, Login, Registro, Reportar, Mis reportes, Ajustes y Crear reporte. Corregido: la pestaña "Mis reportes" ahora se ve entera (se achica para entrar) y no se superpone con la barra de gestos (queda muy cerca, ~2 dp, pero sin tocarla). Sigue cortado: en Crear reporte, el texto de ejemplo del campo Ubicación se ve "Dirección o parad" (falta la última "a") porque comparte la fila con el botón GPS. El resto se agranda y se desplaza bien, sin cortes ni superposiciones. Al terminar volví la letra a 1.0. | Antes: se cortaban "Mis repo…" y "Escribí la direcció…".</t>
+          <t>Tercera prueba 12/10/2026 con letra del sistema al máximo (font_scale 2.0), con vecino1 en Crear reporte: el botón "📍 GPS" quedó debajo del campo Ubicación, a todo el ancho, y el texto de ejemplo "Dirección o parada" se ve entero (campo 371 dp de ancho). Al terminar volví la letra a 1.0. | Repetida el 11/10/2026 con letra del sistema al máximo (font_scale 2.0); recorrí Bienvenida, Login, Registro, Reportar, Mis reportes, Ajustes y Crear reporte. Corregido: la pestaña "Mis reportes" ahora se ve entera (se achica para entrar) y no se superpone con la barra de gestos (queda muy cerca, ~2 dp, pero sin tocarla). Sigue cortado: en Crear reporte, el texto de ejemplo del campo Ubicación se ve "Dirección o parad" (falta la última "a") porque comparte la fila con el botón GPS. El resto se agranda y se desplaza bien, sin cortes ni superposiciones. Al terminar volví la letra a 1.0. | Antes: se cortaban "Mis repo…" y "Escribí la direcció…". | Emulador 11/10/2026 (Claude en VS Code): con letra al máximo se cortaban la pestaña "Mis reportes" y el texto de ejemplo de Ubicación. Corregido en el Cambio N° 36: volver a probar. | Segunda prueba 11/10/2026: las pestañas ya entran; seguía cortado "Dirección o parada" al lado del botón GPS. Corregido en el Cambio N° 37: volver a probar.</t>
         </is>
       </c>
       <c r="M56" s="30" t="inlineStr">
         <is>
-          <t>Claude en VS Code, emulador</t>
+          <t>Claude (automatizado)</t>
         </is>
       </c>
       <c r="N56" s="31" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="57" ht="23.85" customHeight="1" s="21">
@@ -4177,16 +4205,16 @@
       </c>
       <c r="L57" s="30" t="inlineStr">
         <is>
-          <t>Repetida el 11/10/2026: medí con uiautomator (1 dp = 2,625 px) los elementos tocables de Bienvenida, Login, Registro, Reportar, Mis reportes, Ajustes y Crear reporte. Todos cumplen 44 × 44: tema "Claro"/"Oscuro" 168 × 44 dp; "Probar" 44 × 44 dp (115 px, minWidth 44 redondeado al píxel) + hitSlop vertical; "← Volver"/"← Cancelar" 44 dp de alto; campos 45; botones 46-50; pestañas 103 × 49; chips de "¿Qué pasó?" 35 + hitSlop 12 = 47. Fuera del alcance de la corrida anterior, en Mapa NO cumplen: "Paradas y líneas"/"Mapa de calor" y "Filtros del mapa" (40 dp de alto, sin hitSlop; MapaPantalla.tsx líneas 158 y 164) y la "X" de la parada elegida (ícono 22 + hitSlop 10 = 42 dp). | Antes (Falla): tema 40 dp y "Probar" 42 dp de ancho.</t>
+          <t>Tercera prueba 12/10/2026 con letra al máximo, medido con uiautomator en Mapa (1 dp = 2,625 px): "Paradas y líneas" 189,7 × 44,2 dp; "Mapa de calor" 189,7 × 44,2 dp; "Filtros del mapa" 228,6 × 44,2 dp; "X" (Cerrar) de la parada elegida (San Martín y Bolívar) 44,2 × 44,2 dp. Todo ≥ 44. Fuera de lo pedido: los marcadores de parada del mapa miden ~26 dp (son íconos del mapa, no botones de la app), y con la ficha abierta la leyenda "Paradas © colaboradores de OpenStreetMap" queda flotando en medio del mapa. | Repetida el 11/10/2026: medí con uiautomator (1 dp = 2,625 px) los elementos tocables de Bienvenida, Login, Registro, Reportar, Mis reportes, Ajustes y Crear reporte. Todos cumplen 44 × 44: tema "Claro"/"Oscuro" 168 × 44 dp; "Probar" 44 × 44 dp (115 px, minWidth 44 redondeado al píxel) + hitSlop vertical; "← Volver"/"← Cancelar" 44 dp de alto; campos 45; botones 46-50; pestañas 103 × 49; chips de "¿Qué pasó?" 35 + hitSlop 12 = 47. Fuera del alcance de la corrida anterior, en Mapa NO cumplen: "Paradas y líneas"/"Mapa de calor" y "Filtros del mapa" (40 dp de alto, sin hitSlop; MapaPantalla.tsx líneas 158 y 164) y la "X" de la parada elegida (ícono 22 + hitSlop 10 = 42 dp). | Antes (Falla): tema 40 dp y "Probar" 42 dp de ancho. | Emulador 11/10/2026: Claro/Oscuro medían 40 de alto y "Probar" 42 de ancho. Corregido en el Cambio N° 36: volver a probar (falta medir la pantalla Mapa). | Segunda prueba 11/10/2026: Ajustes y "Probar" ya miden 44; en Mapa los botones medían 40 y la X 42. Corregido en el Cambio N° 37: volver a probar. | Se carga Falla porque el criterio es "cualquier pantalla" y Mapa no cumplía.</t>
         </is>
       </c>
       <c r="M57" s="30" t="inlineStr">
         <is>
-          <t>Claude en VS Code, emulador</t>
+          <t>Claude (automatizado)</t>
         </is>
       </c>
       <c r="N57" s="31" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="58" ht="23.85" customHeight="1" s="21">
@@ -4240,21 +4268,21 @@
       </c>
       <c r="K58" s="30" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L58" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 20). | Confirmación de correo y SMTP pospuestos por decisión de emiliano (11/10/2026).</t>
+          <t>Probado 12/10/2026 en la beta con ojoalbondi.app@gmail.com (contraseña de prueba: OjoBondi2026), recién registrada: el registro mostró "Cuenta creada". Al iniciar sesión sin confirmar se mostró "Confirmá tu correo con el mail que te enviamos antes de iniciar sesión." y la app quedó en Login. | Agregado el 11/10/2026 (Registro de cambio N° 20). | Corrección 11/10/2026: en la beta la confirmación de correo SÍ está activa (una cuenta nueva quedó sin confirmar y Supabase reenvió el mail), así que este caso se puede probar. Se quita el Bloqueado.</t>
         </is>
       </c>
       <c r="M58" s="30" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Claude (automatizado)</t>
         </is>
       </c>
       <c r="N58" s="31" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="59" ht="23.85" customHeight="1" s="21">
@@ -4308,21 +4336,21 @@
       </c>
       <c r="K59" s="30" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L59" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 20). | Confirmación de correo y SMTP pospuestos por decisión de emiliano (11/10/2026).</t>
+          <t>Probado 12/10/2026 en la beta con ojoalbondi.app@gmail.com después de confirmar el mail: inició sesión y entró a Reportar ("Hola, Prueba"). Ojo: el enlace del mail de confirmación redirige a localhost:3000 (Site URL por defecto de Supabase) y en el celular abre una página de error "This site can't be reached", aunque la cuenta queda confirmada. Conviene configurar Site URL / Redirect URLs en Supabase &gt; Authentication &gt; URL Configuration. | Agregado el 11/10/2026 (Registro de cambio N° 20). | Corrección 11/10/2026: en la beta la confirmación de correo SÍ está activa (una cuenta nueva quedó sin confirmar y Supabase reenvió el mail), así que este caso se puede probar. Se quita el Bloqueado.</t>
         </is>
       </c>
       <c r="M59" s="30" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Claude (automatizado)</t>
         </is>
       </c>
       <c r="N59" s="31" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="60" ht="23.85" customHeight="1" s="21">
@@ -4947,12 +4975,12 @@
       </c>
       <c r="L69" s="30" t="inlineStr">
         <is>
-          <t>Repetida el 11/10/2026 con el código actualizado: Ajustes de vecino1 muestra Apariencia (Claro/Oscuro), Permisos (Ubicación), Legal (Términos y condiciones) y Cerrar sesión; ya no aparece la sección Notificaciones ni el interruptor "Avisos de estado". | Antes (Falla): la sección NOTIFICACIONES seguía en esta copia porque el cambio N° 32 no estaba aplicado.</t>
+          <t>Agregado el 11/10/2026 (Registro de cambio N° 32). Vuelve cuando se implemente RF-09. | Emulador 11/10/2026: falló porque la carpeta usada no tenía el zip de la revisión de código (Cambio N° 32). Repetir con ese zip aplicado. | Segunda prueba 11/10/2026 con el zip de la revisión aplicado: pasa.</t>
         </is>
       </c>
       <c r="M69" s="30" t="inlineStr">
         <is>
-          <t>Claude en VS Code, emulador</t>
+          <t>Claude en VS Code (emulador)</t>
         </is>
       </c>
       <c r="N69" s="31" t="n">
@@ -5340,6 +5368,132 @@
       </c>
       <c r="M76" s="30" t="n"/>
       <c r="N76" s="31" t="n"/>
+    </row>
+    <row r="77" ht="23.85" customHeight="1" s="21">
+      <c r="A77" s="32" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="33" t="inlineStr">
+        <is>
+          <t>CA-RNF06-3</t>
+        </is>
+      </c>
+      <c r="C77" s="32" t="inlineStr">
+        <is>
+          <t>RNF-06 Accesibilidad</t>
+        </is>
+      </c>
+      <c r="D77" s="32" t="inlineStr">
+        <is>
+          <t>9. Accesibilidad</t>
+        </is>
+      </c>
+      <c r="E77" s="32" t="inlineStr">
+        <is>
+          <t>Cualquiera</t>
+        </is>
+      </c>
+      <c r="F77" s="32" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G77" s="32" t="inlineStr">
+        <is>
+          <t>Estoy en Ajustes (o, con una cuenta de empresa o administración, en Bandeja, Cuentas o Suscripciones)</t>
+        </is>
+      </c>
+      <c r="H77" s="32" t="inlineStr">
+        <is>
+          <t>Desplazo la pantalla hacia abajo</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="inlineStr">
+        <is>
+          <t>El encabezado pasa por debajo de una franja del mismo color; nunca se ve encimado con la hora ni con los íconos de la barra de estado</t>
+        </is>
+      </c>
+      <c r="J77" s="32" t="inlineStr">
+        <is>
+          <t>Probar también con tema oscuro.</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L77" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con letra al máximo, con vecino1 en Ajustes, desplazando hasta que el título pasa por arriba. La barra de estado ocupa y = 0 a 132 px; la franja azul la cubre entera y el título recién se ve desde y = 132, así que nunca se encima con la hora ni con los íconos. Igual en tema claro y oscuro (captura: claro a la izquierda, oscuro a la derecha). Detalle: en tema claro los íconos de la barra de estado se ven oscuros sobre la franja azul oscura (poco contraste); en oscuro se ven blancos. Al terminar volví a tema Claro. | Agregado el 12/10/2026 (Registro de cambio N° 38).</t>
+        </is>
+      </c>
+      <c r="M77" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N77" s="31" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="78" ht="23.85" customHeight="1" s="21">
+      <c r="A78" s="28" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="29" t="inlineStr">
+        <is>
+          <t>CA-RF01-7</t>
+        </is>
+      </c>
+      <c r="C78" s="28" t="inlineStr">
+        <is>
+          <t>RF-01 Registro</t>
+        </is>
+      </c>
+      <c r="D78" s="28" t="inlineStr">
+        <is>
+          <t>1. Registro e inicio de sesión</t>
+        </is>
+      </c>
+      <c r="E78" s="28" t="inlineStr">
+        <is>
+          <t>Correo nuevo (sin cuenta)</t>
+        </is>
+      </c>
+      <c r="F78" s="28" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G78" s="28" t="inlineStr">
+        <is>
+          <t>Supabase ya mandó el máximo de correos de la hora (con el SMTP incluido son 2)</t>
+        </is>
+      </c>
+      <c r="H78" s="28" t="inlineStr">
+        <is>
+          <t>Me registro con un correo nuevo</t>
+        </is>
+      </c>
+      <c r="I78" s="28" t="inlineStr">
+        <is>
+          <t>Se muestra "Se enviaron demasiados correos en poco tiempo. Esperá alrededor de una hora e intentá de nuevo." y la cuenta no se crea</t>
+        </is>
+      </c>
+      <c r="J78" s="28" t="inlineStr">
+        <is>
+          <t>Registrar 3 correos nuevos seguidos; el tercero tiene que mostrar el mensaje.</t>
+        </is>
+      </c>
+      <c r="K78" s="30" t="n"/>
+      <c r="L78" s="30" t="inlineStr">
+        <is>
+          <t>Agregado el 12/10/2026 (Registro de cambio N° 38). Gasta el cupo de correos: dejarlo para después de los casos de mail.</t>
+        </is>
+      </c>
+      <c r="M78" s="30" t="n"/>
+      <c r="N78" s="31" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N300"/>

</xml_diff>

<commit_message>
Pruebas: casos del ciudadano
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
+++ b/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
@@ -1674,10 +1674,24 @@
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
-      <c r="K12" s="30" t="n"/>
-      <c r="L12" s="30" t="n"/>
-      <c r="M12" s="30" t="n"/>
-      <c r="N12" s="31" t="n"/>
+      <c r="K12" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 en la beta con vecino1 (letra 1.0, tema Claro): línea 501, hacia Pilar, Demora/poca frecuencia, interno 1245, descripción "PRUEBA EMULADOR CA-RF03-1", fecha de hoy, 10:30 hs, Parada Bolívar e Ituzaingó (elegida en el mapa). Al tocar "Enviar reporte" pasó a Confirmación con OB-2026-0151; en la base quedó con todos esos datos y la parada vinculada. Captura: formulario (2 partes) y Confirmación.</t>
+        </is>
+      </c>
+      <c r="M12" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N12" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="13" ht="23.85" customHeight="1" s="21">
       <c r="A13" s="32" t="n">
@@ -1724,10 +1738,24 @@
         </is>
       </c>
       <c r="J13" s="32" t="n"/>
-      <c r="K13" s="30" t="n"/>
-      <c r="L13" s="30" t="n"/>
-      <c r="M13" s="30" t="n"/>
-      <c r="N13" s="31" t="n"/>
+      <c r="K13" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L13" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: con el formulario vacío, "Enviar reporte" muestra "Completá línea, sentido, motivo, fecha, horario y ubicación." y queda en Crear reporte. Nota: el mensaje es siempre el mismo, lista todos los obligatorios aunque falte uno solo (no marca cuál falta).</t>
+        </is>
+      </c>
+      <c r="M13" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N13" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" s="21">
       <c r="A14" s="28" t="n">
@@ -1774,10 +1802,24 @@
         </is>
       </c>
       <c r="J14" s="28" t="n"/>
-      <c r="K14" s="30" t="n"/>
-      <c r="L14" s="30" t="n"/>
-      <c r="M14" s="30" t="n"/>
-      <c r="N14" s="31" t="n"/>
+      <c r="K14" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L14" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: con "Robo, hurto o agresión en la parada del colectivo" aparece "🚨 Si estás en peligro o acabás de sufrir un delito, llamá al 911. Este reclamo no reemplaza una denuncia policial." y la etiqueta pasa a "Interno o patente (opcional)". Con el interno vacío se envió (OB-2026-0152, descripción "PRUEBA EMULADOR CA-RF03-3").</t>
+        </is>
+      </c>
+      <c r="M14" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N14" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="15" ht="23.85" customHeight="1" s="21">
       <c r="A15" s="32" t="n">
@@ -1824,10 +1866,24 @@
         </is>
       </c>
       <c r="J15" s="32" t="n"/>
-      <c r="K15" s="30" t="n"/>
-      <c r="L15" s="30" t="n"/>
-      <c r="M15" s="30" t="n"/>
-      <c r="N15" s="31" t="n"/>
+      <c r="K15" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L15" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: con todo completo (501, hacia Pilar, Demora/poca frecuencia, hoy 10:30, "Rivadavia 500, Pilar") y el interno vacío, se muestra "El interno o la patente es obligatorio para este motivo." y no se envía.</t>
+        </is>
+      </c>
+      <c r="M15" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N15" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="16" ht="23.85" customHeight="1" s="21">
       <c r="A16" s="28" t="n">
@@ -1874,10 +1930,24 @@
         </is>
       </c>
       <c r="J16" s="28" t="n"/>
-      <c r="K16" s="30" t="n"/>
-      <c r="L16" s="30" t="n"/>
-      <c r="M16" s="30" t="n"/>
-      <c r="N16" s="31" t="n"/>
+      <c r="K16" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L16" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: con "Hice señas y el colectivo no frenó" se ven la ayuda general ("El número de interno está pintado en el frente, los costados y la parte de atrás del colectivo.") y la adicional en negrita ("Si no frenó, fijate el número en la parte de atrás cuando se aleja.").</t>
+        </is>
+      </c>
+      <c r="M16" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N16" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="21">
       <c r="A17" s="32" t="n">
@@ -1924,10 +1994,24 @@
         </is>
       </c>
       <c r="J17" s="32" t="n"/>
-      <c r="K17" s="30" t="n"/>
-      <c r="L17" s="30" t="n"/>
-      <c r="M17" s="30" t="n"/>
-      <c r="N17" s="31" t="n"/>
+      <c r="K17" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L17" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con la línea 501: Sentido ofrece solo "hacia Pilar", "hacia San Alejo", "hacia Villa Astolfi" y "hacia Villa Rosa", que son los extremos de sus 3 ramales activos en la base (Pilar–Villa Rosa, Pilar–San Alejo, Villa Rosa–Villa Astolfi).</t>
+        </is>
+      </c>
+      <c r="M17" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N17" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="18" ht="35.05" customHeight="1" s="21">
       <c r="A18" s="28" t="n">
@@ -1974,10 +2058,24 @@
         </is>
       </c>
       <c r="J18" s="28" t="n"/>
-      <c r="K18" s="30" t="n"/>
-      <c r="L18" s="30" t="n"/>
-      <c r="M18" s="30" t="n"/>
-      <c r="N18" s="31" t="n"/>
+      <c r="K18" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L18" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: fecha de hoy y 23:30 hs (el emulador marcaba 15:10) → "El horario del hecho no puede ser posterior a la hora actual." y no se envía. Ojo: el emulador está en zona horaria GMT (3 h adelante de Argentina) y la app compara con la hora del celular.</t>
+        </is>
+      </c>
+      <c r="M18" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N18" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="19" ht="35.05" customHeight="1" s="21">
       <c r="A19" s="32" t="n">
@@ -2024,10 +2122,24 @@
         </is>
       </c>
       <c r="J19" s="32" t="n"/>
-      <c r="K19" s="30" t="n"/>
-      <c r="L19" s="30" t="n"/>
-      <c r="M19" s="30" t="n"/>
-      <c r="N19" s="31" t="n"/>
+      <c r="K19" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L19" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: en "Elegir la parada en el mapa" busqué "Lorenzo Lopez 600": el mapa se centró con el pin en Lorenzo López y Rivadavia. Toqué la parada Bolívar e Ituzaingó (visible con "Paradas de la línea 501") y confirmé: Ubicación quedó "Parada Bolívar e Ituzaingó" con el mapa chico de la parada. Detalles: el buscador reemplazó mi texto por "Bernardino Rivadavia 702, Pilar" (la misma esquina, nombrada por la otra calle), y la ficha de esa parada dice "Líneas sin informar" aunque aparece con el filtro de la 501. Captura: búsqueda, parada elegida y formulario.</t>
+        </is>
+      </c>
+      <c r="M19" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N19" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="20" ht="35.05" customHeight="1" s="21">
       <c r="A20" s="28" t="n">
@@ -2074,10 +2186,24 @@
         </is>
       </c>
       <c r="J20" s="28" t="n"/>
-      <c r="K20" s="30" t="n"/>
-      <c r="L20" s="30" t="n"/>
-      <c r="M20" s="30" t="n"/>
-      <c r="N20" s="31" t="n"/>
+      <c r="K20" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L20" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: Confirmación muestra "Reporte enviado", "Ticket N° OB-2026-0151", Línea 501, Motivo, Horario 10:30 hs, Ubicación y Estado "Recibido". En la base el ticket aparece una sola vez (formato OB-AAAA-NNNN).</t>
+        </is>
+      </c>
+      <c r="M20" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N20" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="21">
       <c r="A21" s="32" t="n">
@@ -2124,10 +2250,24 @@
         </is>
       </c>
       <c r="J21" s="32" t="n"/>
-      <c r="K21" s="30" t="n"/>
-      <c r="L21" s="30" t="n"/>
-      <c r="M21" s="30" t="n"/>
-      <c r="N21" s="31" t="n"/>
+      <c r="K21" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L21" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: desde Confirmación, "Ver mis reportes" abre Mis reportes con OB-2026-0151 (12/10/2026, Recibido) primero en la lista.</t>
+        </is>
+      </c>
+      <c r="M21" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N21" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="22" ht="23.85" customHeight="1" s="21">
       <c r="A22" s="28" t="n">
@@ -2174,10 +2314,24 @@
         </is>
       </c>
       <c r="J22" s="28" t="n"/>
-      <c r="K22" s="30" t="n"/>
-      <c r="L22" s="30" t="n"/>
-      <c r="M22" s="30" t="n"/>
-      <c r="N22" s="31" t="n"/>
+      <c r="K22" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L22" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con vecino1: Reportar muestra "Hola, Lucía" y los 3 últimos: OB-2026-0152, OB-2026-0151 y OB-2026-0053.</t>
+        </is>
+      </c>
+      <c r="M22" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N22" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="23" ht="35.05" customHeight="1" s="21">
       <c r="A23" s="32" t="n">
@@ -2224,10 +2378,24 @@
         </is>
       </c>
       <c r="J23" s="32" t="n"/>
-      <c r="K23" s="30" t="n"/>
-      <c r="L23" s="30" t="n"/>
-      <c r="M23" s="30" t="n"/>
-      <c r="N23" s="31" t="n"/>
+      <c r="K23" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L23" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con vecino1: Mis reportes lista 23 reclamos, los mismos 23 que tiene en la base (ninguno de otros usuarios), con su estado (Recibido, En revisión, Atendido), ordenados por fecha de registro del más nuevo al más viejo. Captura: comienzo y final de la lista.</t>
+        </is>
+      </c>
+      <c r="M23" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N23" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="24" ht="23.85" customHeight="1" s="21">
       <c r="A24" s="28" t="n">
@@ -2534,10 +2702,24 @@
           <t>Activar el modo avión para simular la falta de señal.</t>
         </is>
       </c>
-      <c r="K28" s="30" t="n"/>
-      <c r="L28" s="30" t="n"/>
-      <c r="M28" s="30" t="n"/>
-      <c r="N28" s="31" t="n"/>
+      <c r="K28" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L28" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con vecino1 y modo avión activado por adb: Crear reporte muestra "📴 Estás sin conexión: el reporte se guarda igual y se envía cuando vuelva la señal.". Con el reclamo completo (501, hacia Villa Rosa, Exceso de pasajeros, interno 2050, "PRUEBA EMULADOR CA-RF07-1") se mostró "Guardado como borrador" — "Sin conexión: se va a enviar solo cuando vuelva la señal.", estado "Borrador local".</t>
+        </is>
+      </c>
+      <c r="M28" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N28" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="29" ht="23.85" customHeight="1" s="21">
       <c r="A29" s="32" t="n">
@@ -2588,10 +2770,24 @@
           <t>Activar el modo avión para simular la falta de señal.</t>
         </is>
       </c>
-      <c r="K29" s="30" t="n"/>
-      <c r="L29" s="30" t="n"/>
-      <c r="M29" s="30" t="n"/>
-      <c r="N29" s="31" t="n"/>
+      <c r="K29" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L29" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: con el borrador de CA-RF07-1, Mis reportes mostraba "1 borrador(es) esperando conexión para enviarse.". Al desactivar el modo avión se envió solo en ~8 s: apareció primero OB-2026-0153 (Recibido), una sola vez en la base. Detalle: sin conexión, Mis reportes no muestra los reclamos ya enviados, solo el aviso del borrador.</t>
+        </is>
+      </c>
+      <c r="M29" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N29" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="30" ht="23.85" customHeight="1" s="21">
       <c r="A30" s="28" t="n">
@@ -4846,14 +5042,24 @@
         </is>
       </c>
       <c r="J67" s="32" t="n"/>
-      <c r="K67" s="30" t="n"/>
+      <c r="K67" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L67" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
-        </is>
-      </c>
-      <c r="M67" s="30" t="n"/>
-      <c r="N67" s="31" t="n"/>
+          <t>Probado 12/10/2026 con modo avión: reclamo con foto (501, hacia San Alejo, Mal estado de la unidad, "PRUEBA EMULADOR CA-RF07-3 con foto") → "Guardado como borrador" con "Foto adjunta al reporte". Al volver la señal se envió solo como OB-2026-0154; después cerré Expo Go (force-stop) y lo abrí con conexión: en Mis reportes aparece una sola vez (25 reclamos, sin borradores), y en la base hay una sola fila con la foto en Storage (fotos-reclamos, 23 KB). Con tratado@prueba.ojoalbondi (Bandeja) el reclamo muestra la foto. IMPORTANTE: la foto se sacó con la cámara del emulador, no de la galería: "Galería" no abre nada porque en este emulador (Android 15) el selector de fotos del sistema está desactivado (ActivityNotFoundException para PICK_IMAGES); la app no muestra ningún mensaje y en desarrollo sale "Uncaught (in promise) … launchImageLibraryAsync has been rejected". Conviene atrapar ese error y avisar al usuario. | Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
+        </is>
+      </c>
+      <c r="M67" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N67" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="68" ht="23.85" customHeight="1" s="21">
       <c r="A68" s="28" t="n">
@@ -5036,14 +5242,24 @@
           <t>Para provocar el rechazo, como administrador en el SQL Editor: update ramales set activo = false where id = &lt;ramal del sentido&gt;; (después volver a activarlo).</t>
         </is>
       </c>
-      <c r="K70" s="30" t="n"/>
+      <c r="K70" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L70" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 32).</t>
-        </is>
-      </c>
-      <c r="M70" s="30" t="n"/>
-      <c r="N70" s="31" t="n"/>
+          <t>Probado 12/10/2026 con vecino1: con modo avión guardé un borrador (501, hacia San Alejo, "PRUEBA EMULADOR CA-RF07-4"); el equipo desactivó en la beta el ramal 2 (501 Pilar–San Alejo, el único con ese destino). Al volver la señal, Mis reportes mostró "Borrador sin enviar · Línea 501", "Hecho del 12/10/2026 07:50 hs", el motivo "El sentido elegido no corresponde a la línea. Volvé a elegirlo." y los botones Reintentar y Descartar. Descartar pidió confirmación ("Descartar borrador — El reporte no se va a enviar y se borra del celular.", CANCELAR / DESCARTAR) y al confirmar el borrador desapareció; en la base no se creó ningún reclamo. Detalle: el primer intento de envío fue justo al abrir la app mientras volvía el wifi, falló como error de red y el borrador quedó "esperando conexión" sin reintentarse hasta un nuevo cambio de red (activé y desactivé el modo avión). Recordar volver a activar el ramal 2. Captura: borrador esperando, rechazo, confirmación y lista final. | Agregado el 11/10/2026 (Registro de cambio N° 32).</t>
+        </is>
+      </c>
+      <c r="M70" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N70" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="71" ht="23.85" customHeight="1" s="21">
       <c r="A71" s="32" t="n">

</xml_diff>

<commit_message>
Pruebas: empresa, municipio y administración
Incluye el aviso de permiso de ubicación del buscador de paradas
(SelectorParada.tsx), probado como CA-RF03-9 (fila nueva del plan).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
+++ b/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:B37"/>
+  <dimension ref="B1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="20" min="1" max="1"/>
@@ -878,6 +878,13 @@
       <c r="B37" s="26" t="inlineStr">
         <is>
           <t>• Datos de la beta distintos a los de arriba: tratado tiene activas la 501, la 501-503 y la 503; pilarbus la 510; rutabus la 511 pendiente; la 520 no tiene suscripción. Ver las observaciones de CA-RF11-3, CA-RF25-1 y CA-RF25-2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>• CA-RF03-9 (12/10/2026): aviso de permiso de ubicación en el buscador del mapa de paradas (cambio de SelectorParada.tsx posterior al N° 40).</t>
         </is>
       </c>
     </row>
@@ -894,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N78"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="20" min="1" max="1"/>
@@ -2834,10 +2841,24 @@
         </is>
       </c>
       <c r="J30" s="28" t="n"/>
-      <c r="K30" s="30" t="n"/>
-      <c r="L30" s="30" t="n"/>
-      <c r="M30" s="30" t="n"/>
-      <c r="N30" s="31" t="n"/>
+      <c r="K30" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L30" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: tratado@prueba.ojoalbondi inicia sesión y entra a "BANDEJA DE RECLAMOS — Tratado del Pilar — Líneas habilitadas: 501, 501-503, 503".</t>
+        </is>
+      </c>
+      <c r="M30" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N30" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="31" ht="23.85" customHeight="1" s="21">
       <c r="A31" s="32" t="n">
@@ -2884,10 +2905,24 @@
         </is>
       </c>
       <c r="J31" s="32" t="n"/>
-      <c r="K31" s="30" t="n"/>
-      <c r="L31" s="30" t="n"/>
-      <c r="M31" s="30" t="n"/>
-      <c r="N31" s="31" t="n"/>
+      <c r="K31" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L31" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con vecino1: recorrí las 4 pestañas (Reportar, Mapa, Mis reportes, Ajustes) desplazando cada una; en ninguna aparece Bandeja, Cambiar estado, Tomar, Anular, Suscripciones ni Cuentas. Las tarjetas de Mis reportes no abren detalle.</t>
+        </is>
+      </c>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N31" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="32" ht="35.05" customHeight="1" s="21">
       <c r="A32" s="28" t="n">
@@ -2934,10 +2969,24 @@
         </is>
       </c>
       <c r="J32" s="28" t="n"/>
-      <c r="K32" s="30" t="n"/>
-      <c r="L32" s="30" t="n"/>
-      <c r="M32" s="30" t="n"/>
-      <c r="N32" s="31" t="n"/>
+      <c r="K32" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L32" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con tratado, filtro Todos: 31 reclamos (los mismos que tiene en la base), solo de las líneas 501, 501-503 y 503, del más reciente al más viejo, cada uno con ticket, línea, antigüedad ("hoy", "hace N días"), motivo, fecha del hecho y estado. Captura: comienzo y final de la lista.</t>
+        </is>
+      </c>
+      <c r="M32" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N32" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="33" ht="35.05" customHeight="1" s="21">
       <c r="A33" s="32" t="n">
@@ -2988,10 +3037,24 @@
           <t>Los datos de prueba incluyen reclamos de hasta 45 días.</t>
         </is>
       </c>
-      <c r="K33" s="30" t="n"/>
-      <c r="L33" s="30" t="n"/>
-      <c r="M33" s="30" t="n"/>
-      <c r="N33" s="31" t="n"/>
+      <c r="K33" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L33" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con tratado: los Recibido/En revisión de más de 7 días (ej. OB-2026-0010 de 10 días, OB-2026-0081 de 15) tienen borde resaltado y la etiqueta "+7 días"; el Anulado OB-2026-0088 (14 días) y los Atendido OB-2026-0016 y 0117 (15 días) no se resaltan.</t>
+        </is>
+      </c>
+      <c r="M33" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N33" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="34" ht="35.05" customHeight="1" s="21">
       <c r="A34" s="28" t="n">
@@ -3042,14 +3105,24 @@
           <t>Hacerlo durante CA-RF25-5, con la suscripción de Tratado del Pilar suspendida, o crear una cuenta de empresa sin suscripción.</t>
         </is>
       </c>
-      <c r="K34" s="30" t="n"/>
+      <c r="K34" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L34" s="30" t="inlineStr">
         <is>
-          <t>En la beta: usar rutabus@prueba.ojoalbondi (la 511 está pendiente), antes de CA-RNF10-2.</t>
-        </is>
-      </c>
-      <c r="M34" s="30" t="n"/>
-      <c r="N34" s="31" t="n"/>
+          <t>Probado 12/10/2026 en la beta con rutabus@prueba.ojoalbondi (511 pendiente), antes de CA-RNF10-2: la Bandeja dice "Sin líneas habilitadas todavía: el administrador tiene que aprobar la suscripción.", contadores en 0 y "No hay reclamos pendientes."; en Todos: "No hay reclamos asignados.". | En la beta: usar rutabus@prueba.ojoalbondi (la 511 está pendiente), antes de CA-RNF10-2.</t>
+        </is>
+      </c>
+      <c r="M34" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N34" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="35" ht="35.05" customHeight="1" s="21">
       <c r="A35" s="32" t="n">
@@ -3096,10 +3169,24 @@
         </is>
       </c>
       <c r="J35" s="32" t="n"/>
-      <c r="K35" s="30" t="n"/>
-      <c r="L35" s="30" t="n"/>
-      <c r="M35" s="30" t="n"/>
-      <c r="N35" s="31" t="n"/>
+      <c r="K35" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L35" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0117: muestra línea, interno, sentido, motivo, fecha y hora, ubicación, descripción, "Ciudadano: Pablo Ruiz" y el mapa chico con la parada (todo igual a la base). Ningún reclamo de prueba tiene a la vez parada y foto: la foto se vio en OB-2026-0154 (captura de CA-RF07-3, a la derecha). Detalles: las fechas del detalle no llevan cero ("26/9/2026", "1/10/2026") a diferencia del resto de la app ("26/09/2026"), y el mapa chico tiene la etiqueta de accesibilidad "Cambiar la parada en el mapa" aunque la empresa no puede cambiarla.</t>
+        </is>
+      </c>
+      <c r="M35" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N35" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="36" ht="23.85" customHeight="1" s="21">
       <c r="A36" s="28" t="n">
@@ -3146,10 +3233,24 @@
         </is>
       </c>
       <c r="J36" s="28" t="n"/>
-      <c r="K36" s="30" t="n"/>
-      <c r="L36" s="30" t="n"/>
-      <c r="M36" s="30" t="n"/>
-      <c r="N36" s="31" t="n"/>
+      <c r="K36" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L36" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0117 (y 0151, 0154): del ciudadano solo se ve "Ciudadano: Nombre Apellido"; no aparecen correo ni fecha de nacimiento.</t>
+        </is>
+      </c>
+      <c r="M36" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N36" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="37" ht="23.85" customHeight="1" s="21">
       <c r="A37" s="32" t="n">
@@ -3196,14 +3297,24 @@
         </is>
       </c>
       <c r="J37" s="32" t="n"/>
-      <c r="K37" s="30" t="n"/>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L37" s="30" t="inlineStr">
         <is>
-          <t>Apoyo en la base (11/10/2026): cambiar_estado acepta Recibido → En revisión. Falta mirar la pantalla.</t>
-        </is>
-      </c>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0151 (Recibido, reclamo de prueba): bajo "Cambiar estado" solo hay "Tomar (En revisión)" y "Anular". | Apoyo en la base (11/10/2026): cambiar_estado acepta Recibido → En revisión. Falta mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N37" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="38" ht="23.85" customHeight="1" s="21">
       <c r="A38" s="28" t="n">
@@ -3250,14 +3361,24 @@
         </is>
       </c>
       <c r="J38" s="28" t="n"/>
-      <c r="K38" s="30" t="n"/>
+      <c r="K38" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L38" s="30" t="inlineStr">
         <is>
-          <t>Apoyo en la base (11/10/2026): rechaza En revisión → Recibido y acepta En revisión → Atendido. Falta mirar la pantalla.</t>
-        </is>
-      </c>
-      <c r="M38" s="30" t="n"/>
-      <c r="N38" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado: pasé OB-2026-0151 a En revisión (comentario "PRUEBA EMULADOR CA-RF14-2"); ahora solo ofrece "Marcar como Atendido" y "Anular". En la base: Recibido &gt; En revisión. | Apoyo en la base (11/10/2026): rechaza En revisión → Recibido y acepta En revisión → Atendido. Falta mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="M38" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N38" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="39" ht="23.85" customHeight="1" s="21">
       <c r="A39" s="32" t="n">
@@ -3304,14 +3425,24 @@
         </is>
       </c>
       <c r="J39" s="32" t="n"/>
-      <c r="K39" s="30" t="n"/>
+      <c r="K39" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L39" s="30" t="inlineStr">
         <is>
-          <t>Apoyo en la base (11/10/2026): rechaza Atendido → Anulado. Falta mirar la pantalla.</t>
-        </is>
-      </c>
-      <c r="M39" s="30" t="n"/>
-      <c r="N39" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado: OB-2026-0151 marcado Atendido ("PRUEBA EMULADOR CA-RF14-3") y OB-2026-0152 Anulado (motivo "PRUEBA EMULADOR CA-RF14-3"): en los dos, "Cambiar estado" muestra "Estado final: no admite más cambios." sin botones. Solo se cambiaron 0151 y 0152; 0153 y 0154 siguen Recibido. | Apoyo en la base (11/10/2026): rechaza Atendido → Anulado. Falta mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="M39" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N39" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="40" ht="23.85" customHeight="1" s="21">
       <c r="A40" s="28" t="n">
@@ -3358,14 +3489,24 @@
         </is>
       </c>
       <c r="J40" s="28" t="n"/>
-      <c r="K40" s="30" t="n"/>
+      <c r="K40" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L40" s="30" t="inlineStr">
         <is>
-          <t>Apoyo en la base (11/10/2026): anular sin motivo da "El motivo de anulación es obligatorio.". Falta mirar la pantalla.</t>
-        </is>
-      </c>
-      <c r="M40" s="30" t="n"/>
-      <c r="N40" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0152: "Anular" abre "Anular reclamo" (motivos rápidos, campo "Motivo de anulación", Confirmar/Cancelar); al confirmar sin motivo se muestra "El motivo de anulación es obligatorio." y en la base siguió Recibido con una sola entrada. | Apoyo en la base (11/10/2026): anular sin motivo da "El motivo de anulación es obligatorio.". Falta mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="M40" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N40" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="41" ht="46.25" customHeight="1" s="21">
       <c r="A41" s="32" t="n">
@@ -3480,10 +3621,24 @@
         </is>
       </c>
       <c r="J42" s="28" t="n"/>
-      <c r="K42" s="30" t="n"/>
-      <c r="L42" s="30" t="n"/>
-      <c r="M42" s="30" t="n"/>
-      <c r="N42" s="31" t="n"/>
+      <c r="K42" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L42" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0117: Seguimiento muestra en orden Recibido (26/9/2026 20:31, Sistema: reclamo recibido.), En revisión (29/9/2026 02:47, Tratado del Pilar: Estamos revisando...) y Atendido (1/10/2026 12:06, Tratado del Pilar: Se reforzó la frecuencia...), igual que historial_estados.</t>
+        </is>
+      </c>
+      <c r="M42" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N42" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="43" ht="23.85" customHeight="1" s="21">
       <c r="A43" s="32" t="n">
@@ -3530,14 +3685,24 @@
         </is>
       </c>
       <c r="J43" s="32" t="n"/>
-      <c r="K43" s="30" t="n"/>
+      <c r="K43" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L43" s="30" t="inlineStr">
         <is>
-          <t>Apoyo en la base (11/10/2026): un reclamo nuevo tiene una sola entrada, Recibido, registrada por Sistema. Falta mirar la pantalla.</t>
-        </is>
-      </c>
-      <c r="M43" s="30" t="n"/>
-      <c r="N43" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado en OB-2026-0151 recién creado (antes de CA-RF14): una sola entrada, Recibido, 12/10/2026 12:19, "Sistema: reclamo recibido.". | Apoyo en la base (11/10/2026): un reclamo nuevo tiene una sola entrada, Recibido, registrada por Sistema. Falta mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="M43" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N43" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="44" ht="46.25" customHeight="1" s="21">
       <c r="A44" s="28" t="n">
@@ -3584,10 +3749,24 @@
         </is>
       </c>
       <c r="J44" s="28" t="n"/>
-      <c r="K44" s="30" t="n"/>
-      <c r="L44" s="30" t="n"/>
-      <c r="M44" s="30" t="n"/>
-      <c r="N44" s="31" t="n"/>
+      <c r="K44" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L44" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026: los reclamos de la 501 creados por vecino1 (OB-2026-0151 a 0154) aparecen en la Bandeja de Tratado del Pilar; en la de pilarbus (32 reclamos, todos de la 510) no aparece ninguno.</t>
+        </is>
+      </c>
+      <c r="M44" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N44" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="45" ht="23.85" customHeight="1" s="21">
       <c r="A45" s="32" t="n">
@@ -3634,10 +3813,24 @@
         </is>
       </c>
       <c r="J45" s="32" t="n"/>
-      <c r="K45" s="30" t="n"/>
-      <c r="L45" s="30" t="n"/>
-      <c r="M45" s="30" t="n"/>
-      <c r="N45" s="31" t="n"/>
+      <c r="K45" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L45" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con municipio ("Todas las líneas"): en Todos ve 154 reclamos de las 6 líneas (501: 18, 501-503: 8, 503: 5, 510: 32, 511: 10, 520: 81), igual que la base.</t>
+        </is>
+      </c>
+      <c r="M45" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N45" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="46" ht="35.05" customHeight="1" s="21">
       <c r="A46" s="28" t="n">
@@ -3684,14 +3877,24 @@
         </is>
       </c>
       <c r="J46" s="28" t="n"/>
-      <c r="K46" s="30" t="n"/>
+      <c r="K46" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L46" s="30" t="inlineStr">
         <is>
-          <t>En la beta la 503 tiene suscripción activa de Tratado, así que el caso no se da como está escrito. Equivalente en la beta: rutabus opera la 511 con suscripción pendiente y no ve ningún reclamo de la 511.</t>
-        </is>
-      </c>
-      <c r="M46" s="30" t="n"/>
-      <c r="N46" s="31" t="n"/>
+          <t>Probado 12/10/2026 con el equivalente de la beta: rutabus opera la 511 con suscripción pendiente y no ve ninguno de sus 10 reclamos (Pendientes y Todos vacíos). Hecho antes de activar la 511. | En la beta la 503 tiene suscripción activa de Tratado, así que el caso no se da como está escrito. Equivalente en la beta: rutabus opera la 511 con suscripción pendiente y no ve ningún reclamo de la 511.</t>
+        </is>
+      </c>
+      <c r="M46" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N46" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="47" ht="23.85" customHeight="1" s="21">
       <c r="A47" s="32" t="n">
@@ -3742,14 +3945,24 @@
           <t>La 503 no tiene suscripción en los datos de prueba.</t>
         </is>
       </c>
-      <c r="K47" s="30" t="n"/>
+      <c r="K47" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L47" s="30" t="inlineStr">
         <is>
-          <t>En la beta: usar la 520 (sin suscripción) o la 511 (pendiente); el municipio las ve y las gestiona.</t>
-        </is>
-      </c>
-      <c r="M47" s="30" t="n"/>
-      <c r="N47" s="31" t="n"/>
+          <t>Probado 12/10/2026 con municipio y el equivalente de la beta: ve los reclamos de la 520 (sin suscripción, 81) y de la 511 (pendiente, 10) y los puede gestionar: en OB-2026-0053 (520) y OB-2026-0129 (511) aparecen "Tomar (En revisión)" y "Anular" (no se tocaron). | En la beta: usar la 520 (sin suscripción) o la 511 (pendiente); el municipio las ve y las gestiona.</t>
+        </is>
+      </c>
+      <c r="M47" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N47" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="48" ht="46.25" customHeight="1" s="21">
       <c r="A48" s="28" t="n">
@@ -4934,14 +5147,24 @@
         </is>
       </c>
       <c r="J65" s="32" t="n"/>
-      <c r="K65" s="30" t="n"/>
+      <c r="K65" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L65" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
-        </is>
-      </c>
-      <c r="M65" s="30" t="n"/>
-      <c r="N65" s="31" t="n"/>
+          <t>Probado 12/10/2026 con tratado: entré con conexión, cerré Expo Go (force-stop) sin cerrar sesión, activé el modo avión y lo volví a abrir: aparece la Bandeja de Tratado del Pilar (no la pantalla del ciudadano). Como en modo avión Expo Go no puede bajar el código por la red local, el proyecto se abrió como exp://localhost:8081 con adb reverse (Supabase igual sin conexión). Detalle: sin conexión la Bandeja muestra "No se pudieron cargar los reclamos. Revisá tu conexión." pero también "Sin líneas habilitadas todavía: el administrador tiene que aprobar la suscripción." y "No hay reclamos pendientes.", que confunden (no es que no haya, es que no se pudieron cargar). Modo avión desactivado al terminar. | Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
+        </is>
+      </c>
+      <c r="M65" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N65" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="66" ht="23.85" customHeight="1" s="21">
       <c r="A66" s="28" t="n">
@@ -4988,14 +5211,24 @@
         </is>
       </c>
       <c r="J66" s="28" t="n"/>
-      <c r="K66" s="30" t="n"/>
+      <c r="K66" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L66" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
-        </is>
-      </c>
-      <c r="M66" s="30" t="n"/>
-      <c r="N66" s="31" t="n"/>
+          <t>Probado 12/10/2026 con municipio (154 reclamos en Todos, 86 pendientes): en dos vueltas, por cada filtro bajé rápido hasta el final 40 veces, volví arriba y recorrí la lista entera: Pendientes 86/86 y Todos 154/154, sin repetidos y sin Atendidos/Anulados en Pendientes. Cambié entre Pendientes y Todos varias veces. | Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
+        </is>
+      </c>
+      <c r="M66" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N66" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="67" ht="23.85" customHeight="1" s="21">
       <c r="A67" s="32" t="n">
@@ -5364,10 +5597,24 @@
         </is>
       </c>
       <c r="J72" s="28" t="n"/>
-      <c r="K72" s="30" t="n"/>
-      <c r="L72" s="30" t="n"/>
-      <c r="M72" s="30" t="n"/>
-      <c r="N72" s="31" t="n"/>
+      <c r="K72" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L72" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con admin: en Suscripciones la Línea 511 figuraba "Sin suscripción · Opera: Ruta Bus · Gestiona: Municipio" (en la base, pendiente). "Activar suscripción" (empresa Ruta Bus preseleccionada) &gt; Activar: quedó "Suscripción activa · Gestiona: Ruta Bus · desde 12/10/2026", y rutabus ve los 10 reclamos de la 511. Detalle: en la base quedó una fila nueva "activa" y la vieja "pendiente" sigue (dos filas para la 511). Expo Go se cayó (crash del WebView) justo después de activar; la activación ya estaba guardada.</t>
+        </is>
+      </c>
+      <c r="M72" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N72" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="73" ht="23.85" customHeight="1" s="21">
       <c r="A73" s="32" t="n">
@@ -5414,10 +5661,24 @@
         </is>
       </c>
       <c r="J73" s="32" t="n"/>
-      <c r="K73" s="30" t="n"/>
-      <c r="L73" s="30" t="n"/>
-      <c r="M73" s="30" t="n"/>
-      <c r="N73" s="31" t="n"/>
+      <c r="K73" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L73" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con admin: en Cuentas busqué ojoalbondi.app, le puse rol "Empresa de transporte" y organización Pilar Bus, Guardar. Al iniciar sesión con esa cuenta entró a la Bandeja de Pilar Bus (línea 510). Después, desde Cuentas, la volví a Ciudadano (en la base: ciudadano, sin organización).</t>
+        </is>
+      </c>
+      <c r="M73" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N73" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="74" ht="23.85" customHeight="1" s="21">
       <c r="A74" s="28" t="n">
@@ -5464,14 +5725,24 @@
         </is>
       </c>
       <c r="J74" s="28" t="n"/>
-      <c r="K74" s="30" t="n"/>
+      <c r="K74" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L74" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 11/10/2026 (Registro de cambio N° 33).</t>
-        </is>
-      </c>
-      <c r="M74" s="30" t="n"/>
-      <c r="N74" s="31" t="n"/>
+          <t>Probado 12/10/2026 en la beta: vecino1 ve sus reclamos en Mis reportes (25); tratado ve en la Bandeja solo 501, 501-503 y 503 (31); municipio ve todas las líneas (154); admin entra a Administración con las pestañas Suscripciones, Cuentas, Mapa y Ajustes. | Agregado el 11/10/2026 (Registro de cambio N° 33).</t>
+        </is>
+      </c>
+      <c r="M74" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N74" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="75" ht="23.85" customHeight="1" s="21">
       <c r="A75" s="32" t="n">
@@ -5518,14 +5789,24 @@
         </is>
       </c>
       <c r="J75" s="32" t="n"/>
-      <c r="K75" s="30" t="n"/>
+      <c r="K75" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L75" s="30" t="inlineStr">
         <is>
-          <t>Al terminar, suspender la suscripción para dejar los datos como estaban. Cambio N° 33.</t>
-        </is>
-      </c>
-      <c r="M75" s="30" t="n"/>
-      <c r="N75" s="31" t="n"/>
+          <t>Probado 12/10/2026: rutabus tenía la Bandeja vacía; admin activó en Suscripciones la 511 para Ruta Bus y al volver a entrar rutabus ve "Líneas habilitadas: 511" y sus 10 reclamos. Por pedido del equipo, la suscripción de la 511 quedó ACTIVA (no se suspendió al terminar). | Al terminar, suspender la suscripción para dejar los datos como estaban. Cambio N° 33.</t>
+        </is>
+      </c>
+      <c r="M75" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N75" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="76" ht="23.85" customHeight="1" s="21">
       <c r="A76" s="28" t="n">
@@ -5710,6 +5991,74 @@
       </c>
       <c r="M78" s="30" t="n"/>
       <c r="N78" s="31" t="n"/>
+    </row>
+    <row r="79" ht="23.85" customHeight="1" s="21">
+      <c r="A79" s="28" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="29" t="inlineStr">
+        <is>
+          <t>CA-RF03-9</t>
+        </is>
+      </c>
+      <c r="C79" s="28" t="inlineStr">
+        <is>
+          <t>RF-03 Crear reclamo</t>
+        </is>
+      </c>
+      <c r="D79" s="28" t="inlineStr">
+        <is>
+          <t>2. Ciudadano: crear reclamo</t>
+        </is>
+      </c>
+      <c r="E79" s="28" t="inlineStr">
+        <is>
+          <t>vecino1@prueba.ojoalbondi</t>
+        </is>
+      </c>
+      <c r="F79" s="28" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="G79" s="28" t="inlineStr">
+        <is>
+          <t>Expo Go (o la app) no tiene el permiso de ubicación y abrí el mapa de paradas</t>
+        </is>
+      </c>
+      <c r="H79" s="28" t="inlineStr">
+        <is>
+          <t>Busco una calle y altura</t>
+        </is>
+      </c>
+      <c r="I79" s="28" t="inlineStr">
+        <is>
+          <t>Se muestra "Para buscar direcciones, la app necesita el permiso de ubicación." con el botón "Dar permiso"; al darlo, la búsqueda se hace</t>
+        </is>
+      </c>
+      <c r="J79" s="28" t="inlineStr">
+        <is>
+          <t>Quitar el permiso: adb shell pm revoke host.exp.exponent android.permission.ACCESS_FINE_LOCATION (y ACCESS_COARSE_LOCATION). Al terminar, devolver el permiso.</t>
+        </is>
+      </c>
+      <c r="K79" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
+      <c r="L79" s="30" t="inlineStr">
+        <is>
+          <t>Probado 12/10/2026 con vecino1: con el permiso de ubicación de Expo Go quitado (pm revoke), en "Elegir la parada en el mapa" busqué "Lorenzo Lopez 600" y apareció "Para buscar direcciones, la app necesita el permiso de ubicación. También podés mover el mapa y tocar la parada." con el botón "Dar permiso". Al tocarlo se abrió el diálogo de Android; con "While using the app" la búsqueda se hizo sola y el mapa se centró en Lorenzo López y Rivadavia (texto sin cambios). El permiso quedó devuelto. Captura: aviso, diálogo y resultado. | Agregado el 12/10/2026 (cambio de SelectorParada.tsx posterior al Registro de cambio N° 40: aviso de permiso para el buscador).</t>
+        </is>
+      </c>
+      <c r="M79" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N79" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N300"/>

</xml_diff>

<commit_message>
Cambio N° 42: Bandeja sin conexión, fechas, mapa chico y WebView del mapa
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
+++ b/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
@@ -3176,7 +3176,7 @@
       </c>
       <c r="L35" s="30" t="inlineStr">
         <is>
-          <t>Probado 12/10/2026 con tratado en OB-2026-0117: muestra línea, interno, sentido, motivo, fecha y hora, ubicación, descripción, "Ciudadano: Pablo Ruiz" y el mapa chico con la parada (todo igual a la base). Ningún reclamo de prueba tiene a la vez parada y foto: la foto se vio en OB-2026-0154 (captura de CA-RF07-3, a la derecha). Detalles: las fechas del detalle no llevan cero ("26/9/2026", "1/10/2026") a diferencia del resto de la app ("26/09/2026"), y el mapa chico tiene la etiqueta de accesibilidad "Cambiar la parada en el mapa" aunque la empresa no puede cambiarla.</t>
+          <t>Revisión del Cambio N° 42 (12/10/2026, tratado, OB-2026-0117). Fechas: el detalle y el seguimiento salen con dos dígitos: "Fecha y hora del hecho: 26/09/2026 17:25 hs"; seguimiento "26/09/2026 20:31 hs", "29/09/2026 02:47 hs", "01/10/2026 12:06 hs" (captura CA42-2). Mapa chico: uiautomator lo muestra como "Mapa con la ubicación del reclamo", clase ImageView (rol imagen) y enabled=false; tocarlo no hace nada. Detalle: el nodo sigue con clickable=true (lo pone el Pressable aunque esté deshabilitado); si se quiere que no figure como tocable, usar un View cuando no hay onPress (captura CA42-3). WebView del mapa: con vecino1 usé la pestaña Mapa y el selector de paradas de Crear reporte 15 minutos (17:12 a 17:28, 12 ciclos: mover, acercar con doble toque, tocar paradas, buscar direcciones; sin enviar reclamos, la base no tiene reclamos nuevos). Expo Go se cayó 1 vez, a las 17:23:22, en la pestaña Mapa; y otra a las 17:10:53 al cambiar de tratado (detalle con mapa chico) a vecino1, antes de empezar los 15 minutos. Las dos son el mismo crash nativo: SIGTRAP en el hilo MemoryInfra del proceso principal de Expo Go, dentro de libwebviewchromium. No se vio ningún cierre del proceso del renderer del WebView (no hubo mapa en blanco que volviera solo), así que onRenderProcessGone no llegó a actuar: este crash tira toda la app y el arreglo no lo cubre. Captura CA42-4 (pestaña Mapa al terminar). | Probado 12/10/2026 con tratado en OB-2026-0117: muestra línea, interno, sentido, motivo, fecha y hora, ubicación, descripción, "Ciudadano: Pablo Ruiz" y el mapa chico con la parada (todo igual a la base). Ningún reclamo de prueba tiene a la vez parada y foto: la foto se vio en OB-2026-0154 (captura de CA-RF07-3, a la derecha). Detalles: las fechas del detalle no llevan cero ("26/9/2026", "1/10/2026") a diferencia del resto de la app ("26/09/2026"), y el mapa chico tiene la etiqueta de accesibilidad "Cambiar la parada en el mapa" aunque la empresa no puede cambiarla.</t>
         </is>
       </c>
       <c r="M35" s="30" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="L65" s="30" t="inlineStr">
         <is>
-          <t>Probado 12/10/2026 con tratado: entré con conexión, cerré Expo Go (force-stop) sin cerrar sesión, activé el modo avión y lo volví a abrir: aparece la Bandeja de Tratado del Pilar (no la pantalla del ciudadano). Como en modo avión Expo Go no puede bajar el código por la red local, el proyecto se abrió como exp://localhost:8081 con adb reverse (Supabase igual sin conexión). Detalle: sin conexión la Bandeja muestra "No se pudieron cargar los reclamos. Revisá tu conexión." pero también "Sin líneas habilitadas todavía: el administrador tiene que aprobar la suscripción." y "No hay reclamos pendientes.", que confunden (no es que no haya, es que no se pudieron cargar). Modo avión desactivado al terminar. | Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
+          <t>Revisión del Cambio N° 42 (12/10/2026, tratado). Bandeja sin conexión: reabrí la app en modo avión (exp://localhost:8081 con adb reverse) y la Bandeja muestra solo "No se pudieron cargar los reclamos. Revisá tu conexión.", con los contadores en "–"; ya no aparecen "Sin líneas habilitadas…" ni "No hay reclamos pendientes." (tampoco "No hay reclamos asignados." en Todos). Al sacar el modo avión y deslizar para recargar volvieron "Líneas habilitadas: 501, 501-503, 503", los contadores y la lista. Pendientes y Todos miden 116 px = 44 dp de alto (uiautomator, densidad 420). Captura CA42-1 (sin conexión y después de recargar). | Probado 12/10/2026 con tratado: entré con conexión, cerré Expo Go (force-stop) sin cerrar sesión, activé el modo avión y lo volví a abrir: aparece la Bandeja de Tratado del Pilar (no la pantalla del ciudadano). Como en modo avión Expo Go no puede bajar el código por la red local, el proyecto se abrió como exp://localhost:8081 con adb reverse (Supabase igual sin conexión). Detalle: sin conexión la Bandeja muestra "No se pudieron cargar los reclamos. Revisá tu conexión." pero también "Sin líneas habilitadas todavía: el administrador tiene que aprobar la suscripción." y "No hay reclamos pendientes.", que confunden (no es que no haya, es que no se pudieron cargar). Modo avión desactivado al terminar. | Agregado el 11/10/2026 (Registro de cambio N° 30).</t>
         </is>
       </c>
       <c r="M65" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Pruebas: API y límite de correos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
+++ b/documentacion/OjoAlBondi_Plan_de_Pruebas.xlsx
@@ -5543,14 +5543,38 @@
           <t>Con supabase-js: supabase.storage.from("fotos-reclamos").upload("&lt;mi id&gt;/prueba.pdf", archivo, { contentType: "application/pdf" }) → error.</t>
         </is>
       </c>
-      <c r="K71" s="30" t="n"/>
+      <c r="K71" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L71" s="30" t="inlineStr">
         <is>
-          <t>Requiere la migración 009. Agregado el 11/10/2026 (Registro de cambio N° 32). | Base revisada el 11/10/2026: el bucket ya es privado, solo image/jpeg y hasta 5 MB (la migración 009 ya rige en la beta). Falta la subida real, que pasa por la API de Storage: correr pruebas/probar-api.mjs desde VS Code.</t>
-        </is>
-      </c>
-      <c r="M71" s="30" t="n"/>
-      <c r="N71" s="31" t="n"/>
+          <t>Probado 12/10/2026 a las 17:52 con node pruebas/probar-api.mjs contra la beta (salida completa; la hora del final sale en formato de 12 h sin AM/PM):
+✔ Pasa   CA-RF02-1 (API) login vecino1  ·  HTTP 200
+✔ Pasa   CA-RF02-2 (API) contraseña incorrecta  ·  HTTP 400 · Invalid login credentials
+✔ Pasa   CA-RF01-6 alta sin fecha de nacimiento  ·  HTTP 500 · Database error saving new user
+✔ Pasa   CA-RF01-6 alta con fecha futura  ·  HTTP 500 · Database error saving new user
+✔ Pasa   CA-RNF01-1 (API) vecino1 no ve reclamos ajenos  ·  25 propios, 0 ajenos
+✔ Pasa   CA-RNF01-2 (API) tratado no ve la 510  ·  []
+✔ Pasa   CA-RNF01-5 (API) tratado: reclamos vacío, reclamos_gestion con datos  ·  reclamos: 0 · reclamos_gestion: 31
+✔ Pasa   CA-RN02-2 (API) vecino1 intenta cambiar su rol  ·  PATCH HTTP 200 · rol actual: ciudadano
+✔ Pasa   CA-RNF01-3 (API) insert con ticket inventado  ·  HTTP 403 · permission denied for table reclamos
+✔ Pasa   CA-RNF01-4 (API) generar_ticket con sesión  ·  HTTP 403 · generar_ticket() solo se usa desde el trigger de reclamos
+✔ Pasa   CA-RNF01-4 (API) generar_ticket sin sesión  ·  HTTP 401 · permission denied for function generar_ticket
+✔ Pasa   CA-RNF01-7 subir PDF  ·  HTTP 400 · mime type application/pdf is not supported
+✔ Pasa   CA-RNF01-7 subir JPEG de 6 MB  ·  HTTP 400 · The object exceeded the maximum allowed size
+13 comprobaciones · 13 pasan · 0 fallan · 12/10/2026, 05:52:37 | Requiere la migración 009. Agregado el 11/10/2026 (Registro de cambio N° 32). | Base revisada el 11/10/2026: el bucket ya es privado, solo image/jpeg y hasta 5 MB (la migración 009 ya rige en la beta). Falta la subida real, que pasa por la API de Storage: correr pruebas/probar-api.mjs desde VS Code.</t>
+        </is>
+      </c>
+      <c r="M71" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N71" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="72" ht="23.85" customHeight="1" s="21">
       <c r="A72" s="28" t="n">
@@ -5983,14 +6007,24 @@
           <t>Registrar 3 correos nuevos seguidos; el tercero tiene que mostrar el mensaje.</t>
         </is>
       </c>
-      <c r="K78" s="30" t="n"/>
+      <c r="K78" s="30" t="inlineStr">
+        <is>
+          <t>Pasa</t>
+        </is>
+      </c>
       <c r="L78" s="30" t="inlineStr">
         <is>
-          <t>Agregado el 12/10/2026 (Registro de cambio N° 38). Gasta el cupo de correos: dejarlo para después de los casos de mail.</t>
-        </is>
-      </c>
-      <c r="M78" s="30" t="n"/>
-      <c r="N78" s="31" t="n"/>
+          <t>Probado 12/10/2026 en el emulador: registré desde la app, seguidas, ojoalbondi.app+limite1@gmail.com (17:56) y +limite2 (17:59): las dos mostraron "Cuenta creada". Con +limite3 (18:01) apareció "Se enviaron demasiados correos en poco tiempo. Esperá alrededor de una hora e intentá de nuevo." y la cuenta no se creó. Datos: nombre Prueba, apellido Límite, nacimiento 15/10/1995, contraseña Prueba123!. En la base quedaron limite1 y limite2 (ciudadano, sin confirmar; no se abrió ningún mail) y no existe limite3. Captura: "Cuenta creada" de limite1 y el aviso de limite3. | Agregado el 12/10/2026 (Registro de cambio N° 38). Gasta el cupo de correos: dejarlo para después de los casos de mail.</t>
+        </is>
+      </c>
+      <c r="M78" s="30" t="inlineStr">
+        <is>
+          <t>Claude (automatizado)</t>
+        </is>
+      </c>
+      <c r="N78" s="31" t="n">
+        <v>46307</v>
+      </c>
     </row>
     <row r="79" ht="23.85" customHeight="1" s="21">
       <c r="A79" s="28" t="n">

</xml_diff>